<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-16 21:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="488">
   <si>
     <t>50001554 - MAPIMI</t>
   </si>
@@ -5216,7 +5216,7 @@
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46189.87503737268</v>
+        <v>46189.891556296294</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>193</v>
@@ -5252,9 +5252,7 @@
       <c r="R57" s="10"/>
       <c r="S57" s="10"/>
       <c r="T57" s="10"/>
-      <c r="U57" s="11" t="s">
-        <v>54</v>
-      </c>
+      <c r="U57" s="10"/>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
@@ -7990,7 +7988,7 @@
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46189.879227303245</v>
+        <v>46189.891457164355</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>128</v>
@@ -8040,8 +8038,8 @@
       <c r="T107" s="10">
         <v>0</v>
       </c>
-      <c r="U107" s="11" t="s">
-        <v>54</v>
+      <c r="U107" s="12" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-17 16:49 UTC
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2744" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="488">
   <si>
     <t>50001554 - MAPIMI</t>
   </si>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9">
-        <v>46189.872632557875</v>
+        <v>46190.641156666665</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>90</v>
@@ -3525,9 +3525,11 @@
       <c r="B28" s="5">
         <v>46167.55682586806</v>
       </c>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5">
+        <v>46190.64114762731</v>
+      </c>
       <c r="D28" s="5">
-        <v>46183.87119947917</v>
+        <v>46190.641165381945</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>98</v>
@@ -3575,10 +3577,10 @@
         <v>33</v>
       </c>
       <c r="T28" s="6">
-        <v>0</v>
-      </c>
-      <c r="U28" s="11" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="U28" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3903,9 +3905,11 @@
       <c r="B34" s="5">
         <v>46189.87339945602</v>
       </c>
-      <c r="C34" s="6"/>
+      <c r="C34" s="5">
+        <v>46190.64358769676</v>
+      </c>
       <c r="D34" s="5">
-        <v>46189.876154247686</v>
+        <v>46190.643601261574</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>121</v>
@@ -3940,8 +3944,12 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="6"/>
-      <c r="T34" s="6"/>
-      <c r="U34" s="6"/>
+      <c r="T34" s="6">
+        <v>1</v>
+      </c>
+      <c r="U34" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
@@ -3950,9 +3958,11 @@
       <c r="B35" s="9">
         <v>46189.874116527775</v>
       </c>
-      <c r="C35" s="10"/>
+      <c r="C35" s="9">
+        <v>46190.643571747685</v>
+      </c>
       <c r="D35" s="9">
-        <v>46189.87818366898</v>
+        <v>46190.64358837963</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>123</v>
@@ -4000,10 +4010,10 @@
         <v>125</v>
       </c>
       <c r="T35" s="10">
-        <v>0</v>
-      </c>
-      <c r="U35" s="11" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="U35" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -4013,9 +4023,11 @@
       <c r="B36" s="5">
         <v>46189.87428425926</v>
       </c>
-      <c r="C36" s="6"/>
+      <c r="C36" s="5">
+        <v>46190.643442395834</v>
+      </c>
       <c r="D36" s="5">
-        <v>46189.87922747685</v>
+        <v>46190.643529444445</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>127</v>
@@ -4063,10 +4075,10 @@
         <v>125</v>
       </c>
       <c r="T36" s="6">
-        <v>0</v>
-      </c>
-      <c r="U36" s="12" t="s">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="U36" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -4188,7 +4200,7 @@
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="9">
-        <v>46169.8780819213</v>
+        <v>46190.64115600694</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>138</v>
@@ -7988,7 +8000,7 @@
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46189.891457164355</v>
+        <v>46190.64346133102</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>128</v>
@@ -8038,8 +8050,8 @@
       <c r="T107" s="10">
         <v>0</v>
       </c>
-      <c r="U107" s="12" t="s">
-        <v>61</v>
+      <c r="U107" s="11" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-13 14:23 Chile
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -6043,7 +6043,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46167.629188032406</v>
+        <v>46216.68609471065</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>226</v>
@@ -6088,9 +6088,11 @@
       <c r="B71" s="9">
         <v>46167.55708079861</v>
       </c>
-      <c r="C71" s="10"/>
+      <c r="C71" s="9">
+        <v>46216.68608863426</v>
+      </c>
       <c r="D71" s="9">
-        <v>46207.17045002315</v>
+        <v>46216.686107546295</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>229</v>
@@ -6138,10 +6140,10 @@
         <v>108</v>
       </c>
       <c r="T71" s="10">
-        <v>0</v>
-      </c>
-      <c r="U71" s="12" t="s">
-        <v>76</v>
+        <v>1</v>
+      </c>
+      <c r="U71" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -6153,7 +6155,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46211.19534319444</v>
+        <v>46216.68612402778</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>234</v>
@@ -6203,8 +6205,8 @@
       <c r="T72" s="6">
         <v>0</v>
       </c>
-      <c r="U72" s="11" t="s">
-        <v>61</v>
+      <c r="U72" s="12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -6214,9 +6216,11 @@
       <c r="B73" s="9">
         <v>46167.55709181713</v>
       </c>
-      <c r="C73" s="10"/>
+      <c r="C73" s="9">
+        <v>46216.68610497685</v>
+      </c>
       <c r="D73" s="9">
-        <v>46207.17044986111</v>
+        <v>46216.68612113426</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>238</v>
@@ -6264,10 +6268,10 @@
         <v>108</v>
       </c>
       <c r="T73" s="10">
-        <v>0</v>
-      </c>
-      <c r="U73" s="12" t="s">
-        <v>76</v>
+        <v>1</v>
+      </c>
+      <c r="U73" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -6279,7 +6283,7 @@
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46211.19534318287</v>
+        <v>46216.68612297454</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>241</v>
@@ -6329,8 +6333,8 @@
       <c r="T74" s="6">
         <v>0</v>
       </c>
-      <c r="U74" s="11" t="s">
-        <v>61</v>
+      <c r="U74" s="12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -6340,9 +6344,11 @@
       <c r="B75" s="9">
         <v>46167.55715278935</v>
       </c>
-      <c r="C75" s="10"/>
+      <c r="C75" s="9">
+        <v>46216.68611923611</v>
+      </c>
       <c r="D75" s="9">
-        <v>46207.17044987269</v>
+        <v>46216.68613528935</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>244</v>
@@ -6390,10 +6396,10 @@
         <v>108</v>
       </c>
       <c r="T75" s="10">
-        <v>0</v>
-      </c>
-      <c r="U75" s="12" t="s">
-        <v>76</v>
+        <v>1</v>
+      </c>
+      <c r="U75" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6405,7 +6411,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46211.195343217594</v>
+        <v>46216.6861346875</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>245</v>
@@ -6455,8 +6461,8 @@
       <c r="T76" s="6">
         <v>0</v>
       </c>
-      <c r="U76" s="11" t="s">
-        <v>61</v>
+      <c r="U76" s="12" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-03 19:55 UTC
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -6492,7 +6492,7 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46203.50206653935</v>
+        <v>46237.7209872338</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>248</v>
@@ -6541,7 +6541,7 @@
         <v>46203.50206046297</v>
       </c>
       <c r="D78" s="5">
-        <v>46237.57050361111</v>
+        <v>46237.81015790509</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>251</v>
@@ -7543,9 +7543,11 @@
       <c r="B96" s="5">
         <v>46167.5572065625</v>
       </c>
-      <c r="C96" s="6"/>
+      <c r="C96" s="5">
+        <v>46237.7209808912</v>
+      </c>
       <c r="D96" s="5">
-        <v>46224.20563896991</v>
+        <v>46237.72100107639</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>280</v>
@@ -7593,10 +7595,10 @@
         <v>62</v>
       </c>
       <c r="T96" s="6">
-        <v>0</v>
-      </c>
-      <c r="U96" s="12" t="s">
-        <v>78</v>
+        <v>1</v>
+      </c>
+      <c r="U96" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-15 16:39 Chile
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -2647,7 +2647,7 @@
         <v>46248.6791030787</v>
       </c>
       <c r="D12" s="5">
-        <v>46248.67910679398</v>
+        <v>46249.63576609954</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="C148" s="6"/>
       <c r="D148" s="5">
-        <v>46235.18785761574</v>
+        <v>46249.63571710648</v>
       </c>
       <c r="E148" s="6" t="s">
         <v>363</v>
@@ -12331,7 +12331,7 @@
       </c>
       <c r="C184" s="6"/>
       <c r="D184" s="5">
-        <v>46241.20079724537</v>
+        <v>46249.636151377315</v>
       </c>
       <c r="E184" s="6" t="s">
         <v>411</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-29 00:25 UTC
</commit_message>
<xml_diff>
--- a/data/50001554 - MAPIMI.xlsx
+++ b/data/50001554 - MAPIMI.xlsx
@@ -3150,7 +3150,7 @@
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46189.87207028935</v>
+        <v>46262.96165982639</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>74</v>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46199.56372103009</v>
+        <v>46262.962951168985</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>129</v>

</xml_diff>